<commit_message>
Workbook tab 2: What-If Scenarios
Baseline plus nine scenarios driven only by tab 1 names; territory design
vs staffing, year-one/steady-state view, true-up and break-even, guardrails.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MkfgHuEoBecbX8EfBGQPru
</commit_message>
<xml_diff>
--- a/workbook/Commercial_Effectiveness_Model.xlsx
+++ b/workbook/Commercial_Effectiveness_Model.xlsx
@@ -9,8 +9,10 @@
   <sheets>
     <sheet name="Orientation" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="1) Data Entry" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2) What-If Scenarios" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
+    <definedName name="v_baseline_banner">'1) Data Entry'!$F$4</definedName>
     <definedName name="v_scope_business">'1) Data Entry'!$H$11</definedName>
     <definedName name="v_period_start">'1) Data Entry'!$H$12</definedName>
     <definedName name="v_period_end">'1) Data Entry'!$H$13</definedName>
@@ -78,6 +80,8 @@
     <definedName name="v_qualification_definition">'1) Data Entry'!$H$84</definedName>
     <definedName name="v_hiring_approval_rule">'1) Data Entry'!$H$85</definedName>
     <definedName name="v_design_authority">'1) Data Entry'!$H$86</definedName>
+    <definedName name="wi_view">'2) What-If Scenarios'!$B$4</definedName>
+    <definedName name="wi_compare">'2) What-If Scenarios'!$B$5</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'1) Data Entry'!$9:$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -86,13 +90,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="6">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="$#,##0;($#,##0);&quot;-&quot;"/>
     <numFmt numFmtId="166" formatCode="+0%;-0%;0%"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="#,##0.0"/>
     <numFmt numFmtId="169" formatCode="0.0"/>
+    <numFmt numFmtId="170" formatCode="+0%;-0%;&quot;&quot;"/>
+    <numFmt numFmtId="171" formatCode="+0.0%;-0.0%;0.0%"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -228,7 +234,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -355,6 +361,23 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="170" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="171" fontId="4" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -743,7 +766,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:E65"/>
+  <dimension ref="B2:E66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -872,10 +895,10 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="31" customHeight="1">
+    <row r="23" ht="44.5" customHeight="1">
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>3.  Explore what-if scenarios (later tabs). Change assumptions one at a time or in combination: territory design, hiring and fill speed, salesperson capacity, win rate, cycle, deal size, costs. Every change flows through to operating income, with nothing unexplained.</t>
+          <t>3.  Explore what-if scenarios (2) What-If Scenarios). Each column is a scenario you can rename and change: territory design, filling open territories, fill speed, ramp, salesperson capacity, opportunities held, win rate, cycle, deal size, costs and the cost of the improvement itself. Every change flows through to operating income, and a true-up row confirms nothing is unexplained.</t>
         </is>
       </c>
     </row>
@@ -1282,33 +1305,40 @@
     <row r="61" ht="31" customHeight="1">
       <c r="B61" s="4" t="inlineStr">
         <is>
-          <t>•  Later tabs (to be rebuilt): performance breakdown, impact on the income statement, scenario diagnostics. They read only the Value used cells on tab 1.</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="17.5" customHeight="1">
-      <c r="B63" s="3" t="inlineStr">
+          <t>•  2) What-If Scenarios: baseline plus nine editable scenarios, from territory design and staffing through salesperson throughput to operating income, with a true-up and a break-even budget for each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="17.5" customHeight="1">
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>•  Later tabs (to be rebuilt): detailed income statement and scenario diagnostics. Every tab reads only the Value used cells on tab 1.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="17.5" customHeight="1">
+      <c r="B64" s="3" t="inlineStr">
         <is>
           <t>A few points</t>
         </is>
       </c>
     </row>
-    <row r="64" ht="31" customHeight="1">
-      <c r="B64" s="4" t="inlineStr">
+    <row r="65" ht="31" customHeight="1">
+      <c r="B65" s="4" t="inlineStr">
         <is>
           <t>This is a general model. For a sharper analysis, run it separately for each sales channel and product line, and separate new-customer revenue from revenue from existing customers. The model can be tailored to your business.</t>
         </is>
       </c>
     </row>
-    <row r="65" ht="44.5" customHeight="1">
-      <c r="B65" s="4" t="inlineStr">
+    <row r="66" ht="44.5" customHeight="1">
+      <c r="B66" s="4" t="inlineStr">
         <is>
           <t>“Increase leads” is not listed as a business scenario because we consider lead generation to be a more leveraged way to conduct sales prospecting. The number of leads, how to acquire them, and how much you can invest to acquire those leads are all handled in the tactical “drill down” spreadsheets that accompany this model.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="39">
+  <mergeCells count="40">
     <mergeCell ref="B65:E65"/>
     <mergeCell ref="B37:E37"/>
     <mergeCell ref="B6:E6"/>
@@ -1318,14 +1348,15 @@
     <mergeCell ref="B24:E24"/>
     <mergeCell ref="B20:E20"/>
     <mergeCell ref="B32:E32"/>
-    <mergeCell ref="B63:E63"/>
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B35:E35"/>
     <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B62:E62"/>
     <mergeCell ref="B7:E7"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="B59:E59"/>
     <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B66:E66"/>
     <mergeCell ref="B18:E18"/>
     <mergeCell ref="B27:E27"/>
     <mergeCell ref="B43:E43"/>
@@ -6661,4 +6692,3015 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:M76"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="17" customWidth="1" min="9" max="9"/>
+    <col width="17" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>2) What-If Scenarios</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="14" t="inlineStr">
+        <is>
+          <t>Each column is a scenario built on the tab 1 baseline. Rename it, describe the question, and enter changes in the yellow cells (blank means no change). Everything below is calculated from tab 1's Value used cells.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="16">
+        <f>v_baseline_banner</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>View</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Year one</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Compare break-even against</t>
+        </is>
+      </c>
+      <c r="B5" s="15" t="inlineStr">
+        <is>
+          <t>Add territories +10%</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>How it works</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Baseline</t>
+        </is>
+      </c>
+      <c r="E7" s="19" t="inlineStr">
+        <is>
+          <t>Add territories +10%</t>
+        </is>
+      </c>
+      <c r="F7" s="19" t="inlineStr">
+        <is>
+          <t>Fill open territories</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>Close rate +10%</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>Cycle −10%</t>
+        </is>
+      </c>
+      <c r="I7" s="19" t="inlineStr">
+        <is>
+          <t>Deal size +10%</t>
+        </is>
+      </c>
+      <c r="J7" s="19" t="inlineStr">
+        <is>
+          <t>Opportunities held +10%</t>
+        </is>
+      </c>
+      <c r="K7" s="19" t="inlineStr">
+        <is>
+          <t>Close, cycle and deal size</t>
+        </is>
+      </c>
+      <c r="L7" s="19" t="inlineStr">
+        <is>
+          <t>All four with territories</t>
+        </is>
+      </c>
+      <c r="M7" s="19" t="inlineStr">
+        <is>
+          <t>Your scenario</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="54" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>Question it answers</t>
+        </is>
+      </c>
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>Tab 1, as entered</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>What if we fund 10% more territories and hire into them?</t>
+        </is>
+      </c>
+      <c r="F8" s="26" t="inlineStr">
+        <is>
+          <t>What if we fill every open territory this year?</t>
+        </is>
+      </c>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>What if we close 10% more of the opportunities we work?</t>
+        </is>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>What if deals take 10% less time?</t>
+        </is>
+      </c>
+      <c r="I8" s="26" t="inlineStr">
+        <is>
+          <t>What if each contract is worth 10% more?</t>
+        </is>
+      </c>
+      <c r="J8" s="26" t="inlineStr">
+        <is>
+          <t>What if 10% more qualified opportunities reach each salesperson?</t>
+        </is>
+      </c>
+      <c r="K8" s="26" t="inlineStr">
+        <is>
+          <t>What if all three quality levers improve 10%?</t>
+        </is>
+      </c>
+      <c r="L8" s="26" t="inlineStr">
+        <is>
+          <t>What if we add territories and improve all three quality levers?</t>
+        </is>
+      </c>
+      <c r="M8" s="26" t="inlineStr">
+        <is>
+          <t>Describe the question this scenario answers</t>
+        </is>
+      </c>
+    </row>
+    <row r="9"/>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>Changes from baseline (blank means no change)</t>
+        </is>
+      </c>
+      <c r="B10" s="21" t="n"/>
+      <c r="D10" s="21" t="n"/>
+      <c r="E10" s="21" t="n"/>
+      <c r="F10" s="21" t="n"/>
+      <c r="G10" s="21" t="n"/>
+      <c r="H10" s="21" t="n"/>
+      <c r="I10" s="21" t="n"/>
+      <c r="J10" s="21" t="n"/>
+      <c r="K10" s="21" t="n"/>
+      <c r="L10" s="21" t="n"/>
+      <c r="M10" s="21" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Funded territories</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Territory design: how many territories the company funds · leverage point 10</t>
+        </is>
+      </c>
+      <c r="D11" s="8" t="n"/>
+      <c r="E11" s="52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F11" s="52" t="n"/>
+      <c r="G11" s="52" t="n"/>
+      <c r="H11" s="52" t="n"/>
+      <c r="I11" s="52" t="n"/>
+      <c r="J11" s="52" t="n"/>
+      <c r="K11" s="52" t="n"/>
+      <c r="L11" s="52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M11" s="52" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Open territories filled</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Staffing: open territories filled during the year (up to the number open) · leverage point 10</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="n"/>
+      <c r="E12" s="53" t="n"/>
+      <c r="F12" s="53">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="G12" s="53" t="n"/>
+      <c r="H12" s="53" t="n"/>
+      <c r="I12" s="53" t="n"/>
+      <c r="J12" s="53" t="n"/>
+      <c r="K12" s="53" t="n"/>
+      <c r="L12" s="53" t="n"/>
+      <c r="M12" s="53" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Days to fill a territory</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Delay: approvals and recruiting · leverage point 9</t>
+        </is>
+      </c>
+      <c r="D13" s="8" t="n"/>
+      <c r="E13" s="52" t="n"/>
+      <c r="F13" s="52" t="n"/>
+      <c r="G13" s="52" t="n"/>
+      <c r="H13" s="52" t="n"/>
+      <c r="I13" s="52" t="n"/>
+      <c r="J13" s="52" t="n"/>
+      <c r="K13" s="52" t="n"/>
+      <c r="L13" s="52" t="n"/>
+      <c r="M13" s="52" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Ramp time</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Delay: months until a new salesperson is fully productive · leverage point 9</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="n"/>
+      <c r="E14" s="52" t="n"/>
+      <c r="F14" s="52" t="n"/>
+      <c r="G14" s="52" t="n"/>
+      <c r="H14" s="52" t="n"/>
+      <c r="I14" s="52" t="n"/>
+      <c r="J14" s="52" t="n"/>
+      <c r="K14" s="52" t="n"/>
+      <c r="L14" s="52" t="n"/>
+      <c r="M14" s="52" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>Opportunities a salesperson can manage</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Capacity: how many opportunities a salesperson can hold and advance well · leverage point 12</t>
+        </is>
+      </c>
+      <c r="D15" s="8" t="n"/>
+      <c r="E15" s="52" t="n"/>
+      <c r="F15" s="52" t="n"/>
+      <c r="G15" s="52" t="n"/>
+      <c r="H15" s="52" t="n"/>
+      <c r="I15" s="52" t="n"/>
+      <c r="J15" s="52" t="n"/>
+      <c r="K15" s="52" t="n"/>
+      <c r="L15" s="52" t="n"/>
+      <c r="M15" s="52" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>Opportunities each salesperson holds</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Pipeline: qualified opportunities reaching salespeople (needs pipeline data on tab 1) · leverage point 11</t>
+        </is>
+      </c>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="52" t="n"/>
+      <c r="F16" s="52" t="n"/>
+      <c r="G16" s="52" t="n"/>
+      <c r="H16" s="52" t="n"/>
+      <c r="I16" s="52" t="n"/>
+      <c r="J16" s="52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K16" s="52" t="n"/>
+      <c r="L16" s="52" t="n"/>
+      <c r="M16" s="52" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Sales cycle</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Delay: time from qualified opportunity to signature · leverage point 9</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="52" t="n"/>
+      <c r="F17" s="52" t="n"/>
+      <c r="G17" s="52" t="n"/>
+      <c r="H17" s="52" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="I17" s="52" t="n"/>
+      <c r="J17" s="52" t="n"/>
+      <c r="K17" s="52" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="L17" s="52" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="M17" s="52" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Close rate</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Conversion · leverage point 12</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="52" t="n"/>
+      <c r="F18" s="52" t="n"/>
+      <c r="G18" s="52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H18" s="52" t="n"/>
+      <c r="I18" s="52" t="n"/>
+      <c r="J18" s="52" t="n"/>
+      <c r="K18" s="52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L18" s="52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M18" s="52" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>Average revenue per contract</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Value per contract · leverage point 12</t>
+        </is>
+      </c>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="52" t="n"/>
+      <c r="F19" s="52" t="n"/>
+      <c r="G19" s="52" t="n"/>
+      <c r="H19" s="52" t="n"/>
+      <c r="I19" s="52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J19" s="52" t="n"/>
+      <c r="K19" s="52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L19" s="52" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M19" s="52" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>Salesperson compensation (salary and load)</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Cost per salesperson · leverage point 12</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="52" t="n"/>
+      <c r="F20" s="52" t="n"/>
+      <c r="G20" s="52" t="n"/>
+      <c r="H20" s="52" t="n"/>
+      <c r="I20" s="52" t="n"/>
+      <c r="J20" s="52" t="n"/>
+      <c r="K20" s="52" t="n"/>
+      <c r="L20" s="52" t="n"/>
+      <c r="M20" s="52" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>Commission rate</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Rule: compensation plan · leverage point 5</t>
+        </is>
+      </c>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="52" t="n"/>
+      <c r="F21" s="52" t="n"/>
+      <c r="G21" s="52" t="n"/>
+      <c r="H21" s="52" t="n"/>
+      <c r="I21" s="52" t="n"/>
+      <c r="J21" s="52" t="n"/>
+      <c r="K21" s="52" t="n"/>
+      <c r="L21" s="52" t="n"/>
+      <c r="M21" s="52" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Sales overhead</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Change in dollars · leverage point 12</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="n"/>
+      <c r="E22" s="54" t="n"/>
+      <c r="F22" s="54" t="n"/>
+      <c r="G22" s="54" t="n"/>
+      <c r="H22" s="54" t="n"/>
+      <c r="I22" s="54" t="n"/>
+      <c r="J22" s="54" t="n"/>
+      <c r="K22" s="54" t="n"/>
+      <c r="L22" s="54" t="n"/>
+      <c r="M22" s="54" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Change in dollars · leverage point 12</t>
+        </is>
+      </c>
+      <c r="D23" s="8" t="n"/>
+      <c r="E23" s="54" t="n"/>
+      <c r="F23" s="54" t="n"/>
+      <c r="G23" s="54" t="n"/>
+      <c r="H23" s="54" t="n"/>
+      <c r="I23" s="54" t="n"/>
+      <c r="J23" s="54" t="n"/>
+      <c r="K23" s="54" t="n"/>
+      <c r="L23" s="54" t="n"/>
+      <c r="M23" s="54" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>Cost of making the change (one-time)</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Enablement, tools, hiring, consulting: what the improvement costs this year · leverage point 12</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="n"/>
+      <c r="E24" s="54" t="n"/>
+      <c r="F24" s="54" t="n"/>
+      <c r="G24" s="54" t="n"/>
+      <c r="H24" s="54" t="n"/>
+      <c r="I24" s="54" t="n"/>
+      <c r="J24" s="54" t="n"/>
+      <c r="K24" s="54" t="n"/>
+      <c r="L24" s="54" t="n"/>
+      <c r="M24" s="54" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="20" t="inlineStr">
+        <is>
+          <t>Territory design and staffing</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="n"/>
+      <c r="D26" s="21" t="n"/>
+      <c r="E26" s="21" t="n"/>
+      <c r="F26" s="21" t="n"/>
+      <c r="G26" s="21" t="n"/>
+      <c r="H26" s="21" t="n"/>
+      <c r="I26" s="21" t="n"/>
+      <c r="J26" s="21" t="n"/>
+      <c r="K26" s="21" t="n"/>
+      <c r="L26" s="21" t="n"/>
+      <c r="M26" s="21" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="7" t="inlineStr">
+        <is>
+          <t>Funded territories</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 funded territories × change</t>
+        </is>
+      </c>
+      <c r="D27" s="55">
+        <f>v_territory_count*(1+D11)</f>
+        <v/>
+      </c>
+      <c r="E27" s="55">
+        <f>v_territory_count*(1+E11)</f>
+        <v/>
+      </c>
+      <c r="F27" s="55">
+        <f>v_territory_count*(1+F11)</f>
+        <v/>
+      </c>
+      <c r="G27" s="55">
+        <f>v_territory_count*(1+G11)</f>
+        <v/>
+      </c>
+      <c r="H27" s="55">
+        <f>v_territory_count*(1+H11)</f>
+        <v/>
+      </c>
+      <c r="I27" s="55">
+        <f>v_territory_count*(1+I11)</f>
+        <v/>
+      </c>
+      <c r="J27" s="55">
+        <f>v_territory_count*(1+J11)</f>
+        <v/>
+      </c>
+      <c r="K27" s="55">
+        <f>v_territory_count*(1+K11)</f>
+        <v/>
+      </c>
+      <c r="L27" s="55">
+        <f>v_territory_count*(1+L11)</f>
+        <v/>
+      </c>
+      <c r="M27" s="55">
+        <f>v_territory_count*(1+M11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Open territories at start</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 (0 if not provided)</t>
+        </is>
+      </c>
+      <c r="D28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="E28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="F28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="G28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="H28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="I28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="J28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="K28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="L28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+      <c r="M28" s="55">
+        <f>N(v_open_territories)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="7" t="inlineStr">
+        <is>
+          <t>Filled territories at start</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>Funded − open</t>
+        </is>
+      </c>
+      <c r="D29" s="55">
+        <f>v_territory_count-D28</f>
+        <v/>
+      </c>
+      <c r="E29" s="55">
+        <f>v_territory_count-E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="55">
+        <f>v_territory_count-F28</f>
+        <v/>
+      </c>
+      <c r="G29" s="55">
+        <f>v_territory_count-G28</f>
+        <v/>
+      </c>
+      <c r="H29" s="55">
+        <f>v_territory_count-H28</f>
+        <v/>
+      </c>
+      <c r="I29" s="55">
+        <f>v_territory_count-I28</f>
+        <v/>
+      </c>
+      <c r="J29" s="55">
+        <f>v_territory_count-J28</f>
+        <v/>
+      </c>
+      <c r="K29" s="55">
+        <f>v_territory_count-K28</f>
+        <v/>
+      </c>
+      <c r="L29" s="55">
+        <f>v_territory_count-L28</f>
+        <v/>
+      </c>
+      <c r="M29" s="55">
+        <f>v_territory_count-M28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>New territories added</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>Design change</t>
+        </is>
+      </c>
+      <c r="D30" s="55">
+        <f>D27-v_territory_count</f>
+        <v/>
+      </c>
+      <c r="E30" s="55">
+        <f>E27-v_territory_count</f>
+        <v/>
+      </c>
+      <c r="F30" s="55">
+        <f>F27-v_territory_count</f>
+        <v/>
+      </c>
+      <c r="G30" s="55">
+        <f>G27-v_territory_count</f>
+        <v/>
+      </c>
+      <c r="H30" s="55">
+        <f>H27-v_territory_count</f>
+        <v/>
+      </c>
+      <c r="I30" s="55">
+        <f>I27-v_territory_count</f>
+        <v/>
+      </c>
+      <c r="J30" s="55">
+        <f>J27-v_territory_count</f>
+        <v/>
+      </c>
+      <c r="K30" s="55">
+        <f>K27-v_territory_count</f>
+        <v/>
+      </c>
+      <c r="L30" s="55">
+        <f>L27-v_territory_count</f>
+        <v/>
+      </c>
+      <c r="M30" s="55">
+        <f>M27-v_territory_count</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="7" t="inlineStr">
+        <is>
+          <t>Open territories filled</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>Up to the number open</t>
+        </is>
+      </c>
+      <c r="D31" s="55">
+        <f>MIN(N(D12),D28)</f>
+        <v/>
+      </c>
+      <c r="E31" s="55">
+        <f>MIN(N(E12),E28)</f>
+        <v/>
+      </c>
+      <c r="F31" s="55">
+        <f>MIN(N(F12),F28)</f>
+        <v/>
+      </c>
+      <c r="G31" s="55">
+        <f>MIN(N(G12),G28)</f>
+        <v/>
+      </c>
+      <c r="H31" s="55">
+        <f>MIN(N(H12),H28)</f>
+        <v/>
+      </c>
+      <c r="I31" s="55">
+        <f>MIN(N(I12),I28)</f>
+        <v/>
+      </c>
+      <c r="J31" s="55">
+        <f>MIN(N(J12),J28)</f>
+        <v/>
+      </c>
+      <c r="K31" s="55">
+        <f>MIN(N(K12),K28)</f>
+        <v/>
+      </c>
+      <c r="L31" s="55">
+        <f>MIN(N(L12),L28)</f>
+        <v/>
+      </c>
+      <c r="M31" s="55">
+        <f>MIN(N(M12),M28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>Territories still open</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>Each one is expected yield not produced</t>
+        </is>
+      </c>
+      <c r="D32" s="55">
+        <f>D28-D31</f>
+        <v/>
+      </c>
+      <c r="E32" s="55">
+        <f>E28-E31</f>
+        <v/>
+      </c>
+      <c r="F32" s="55">
+        <f>F28-F31</f>
+        <v/>
+      </c>
+      <c r="G32" s="55">
+        <f>G28-G31</f>
+        <v/>
+      </c>
+      <c r="H32" s="55">
+        <f>H28-H31</f>
+        <v/>
+      </c>
+      <c r="I32" s="55">
+        <f>I28-I31</f>
+        <v/>
+      </c>
+      <c r="J32" s="55">
+        <f>J28-J31</f>
+        <v/>
+      </c>
+      <c r="K32" s="55">
+        <f>K28-K31</f>
+        <v/>
+      </c>
+      <c r="L32" s="55">
+        <f>L28-L31</f>
+        <v/>
+      </c>
+      <c r="M32" s="55">
+        <f>M28-M31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="7" t="inlineStr">
+        <is>
+          <t>Months to fill a territory</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 days ÷ 30.4 × change</t>
+        </is>
+      </c>
+      <c r="D33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+D13)</f>
+        <v/>
+      </c>
+      <c r="E33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+E13)</f>
+        <v/>
+      </c>
+      <c r="F33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+F13)</f>
+        <v/>
+      </c>
+      <c r="G33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+G13)</f>
+        <v/>
+      </c>
+      <c r="H33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+H13)</f>
+        <v/>
+      </c>
+      <c r="I33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+I13)</f>
+        <v/>
+      </c>
+      <c r="J33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+J13)</f>
+        <v/>
+      </c>
+      <c r="K33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+K13)</f>
+        <v/>
+      </c>
+      <c r="L33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+L13)</f>
+        <v/>
+      </c>
+      <c r="M33" s="56">
+        <f>N(v_time_to_fill_days)/30.4*(1+M13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="7" t="inlineStr">
+        <is>
+          <t>Ramp time (months)</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 × change</t>
+        </is>
+      </c>
+      <c r="D34" s="56">
+        <f>v_ramp_months*(1+D14)</f>
+        <v/>
+      </c>
+      <c r="E34" s="56">
+        <f>v_ramp_months*(1+E14)</f>
+        <v/>
+      </c>
+      <c r="F34" s="56">
+        <f>v_ramp_months*(1+F14)</f>
+        <v/>
+      </c>
+      <c r="G34" s="56">
+        <f>v_ramp_months*(1+G14)</f>
+        <v/>
+      </c>
+      <c r="H34" s="56">
+        <f>v_ramp_months*(1+H14)</f>
+        <v/>
+      </c>
+      <c r="I34" s="56">
+        <f>v_ramp_months*(1+I14)</f>
+        <v/>
+      </c>
+      <c r="J34" s="56">
+        <f>v_ramp_months*(1+J14)</f>
+        <v/>
+      </c>
+      <c r="K34" s="56">
+        <f>v_ramp_months*(1+K14)</f>
+        <v/>
+      </c>
+      <c r="L34" s="56">
+        <f>v_ramp_months*(1+L14)</f>
+        <v/>
+      </c>
+      <c r="M34" s="56">
+        <f>v_ramp_months*(1+M14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>Share of year a newly staffed territory produces</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Year one: (12 − fill − ramp) ÷ 12; steady state: 1</t>
+        </is>
+      </c>
+      <c r="D35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-D33-D34)/12)</f>
+        <v/>
+      </c>
+      <c r="E35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-E33-E34)/12)</f>
+        <v/>
+      </c>
+      <c r="F35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-F33-F34)/12)</f>
+        <v/>
+      </c>
+      <c r="G35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-G33-G34)/12)</f>
+        <v/>
+      </c>
+      <c r="H35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-H33-H34)/12)</f>
+        <v/>
+      </c>
+      <c r="I35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-I33-I34)/12)</f>
+        <v/>
+      </c>
+      <c r="J35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-J33-J34)/12)</f>
+        <v/>
+      </c>
+      <c r="K35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-K33-K34)/12)</f>
+        <v/>
+      </c>
+      <c r="L35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-L33-L34)/12)</f>
+        <v/>
+      </c>
+      <c r="M35" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-M33-M34)/12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="7" t="inlineStr">
+        <is>
+          <t>Share of year a new salesperson is paid</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>Year one: (12 − fill) ÷ 12; steady state: 1</t>
+        </is>
+      </c>
+      <c r="D36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-D33)/12)</f>
+        <v/>
+      </c>
+      <c r="E36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-E33)/12)</f>
+        <v/>
+      </c>
+      <c r="F36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-F33)/12)</f>
+        <v/>
+      </c>
+      <c r="G36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-G33)/12)</f>
+        <v/>
+      </c>
+      <c r="H36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-H33)/12)</f>
+        <v/>
+      </c>
+      <c r="I36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-I33)/12)</f>
+        <v/>
+      </c>
+      <c r="J36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-J33)/12)</f>
+        <v/>
+      </c>
+      <c r="K36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-K33)/12)</f>
+        <v/>
+      </c>
+      <c r="L36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-L33)/12)</f>
+        <v/>
+      </c>
+      <c r="M36" s="57">
+        <f>IF(wi_view="Steady state",1,MAX(0,12-M33)/12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="7" t="inlineStr">
+        <is>
+          <t>Productive salespeople in filled territories</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 productive salespeople, if provided</t>
+        </is>
+      </c>
+      <c r="D37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(D29,v_productive_salespeople),D29)</f>
+        <v/>
+      </c>
+      <c r="E37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(E29,v_productive_salespeople),E29)</f>
+        <v/>
+      </c>
+      <c r="F37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(F29,v_productive_salespeople),F29)</f>
+        <v/>
+      </c>
+      <c r="G37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(G29,v_productive_salespeople),G29)</f>
+        <v/>
+      </c>
+      <c r="H37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(H29,v_productive_salespeople),H29)</f>
+        <v/>
+      </c>
+      <c r="I37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(I29,v_productive_salespeople),I29)</f>
+        <v/>
+      </c>
+      <c r="J37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(J29,v_productive_salespeople),J29)</f>
+        <v/>
+      </c>
+      <c r="K37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(K29,v_productive_salespeople),K29)</f>
+        <v/>
+      </c>
+      <c r="L37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(L29,v_productive_salespeople),L29)</f>
+        <v/>
+      </c>
+      <c r="M37" s="55">
+        <f>IF(N(v_productive_salespeople)&gt;0,MIN(M29,v_productive_salespeople),M29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>Productive territory-years</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>What actually produces revenue this year</t>
+        </is>
+      </c>
+      <c r="D38" s="55">
+        <f>D37+(D31+D30)*D35</f>
+        <v/>
+      </c>
+      <c r="E38" s="55">
+        <f>E37+(E31+E30)*E35</f>
+        <v/>
+      </c>
+      <c r="F38" s="55">
+        <f>F37+(F31+F30)*F35</f>
+        <v/>
+      </c>
+      <c r="G38" s="55">
+        <f>G37+(G31+G30)*G35</f>
+        <v/>
+      </c>
+      <c r="H38" s="55">
+        <f>H37+(H31+H30)*H35</f>
+        <v/>
+      </c>
+      <c r="I38" s="55">
+        <f>I37+(I31+I30)*I35</f>
+        <v/>
+      </c>
+      <c r="J38" s="55">
+        <f>J37+(J31+J30)*J35</f>
+        <v/>
+      </c>
+      <c r="K38" s="55">
+        <f>K37+(K31+K30)*K35</f>
+        <v/>
+      </c>
+      <c r="L38" s="55">
+        <f>L37+(L31+L30)*L35</f>
+        <v/>
+      </c>
+      <c r="M38" s="55">
+        <f>M37+(M31+M30)*M35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="7" t="inlineStr">
+        <is>
+          <t>Salesperson-years paid</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>What the company pays for this year</t>
+        </is>
+      </c>
+      <c r="D39" s="55">
+        <f>D29+(D31+D30)*D36</f>
+        <v/>
+      </c>
+      <c r="E39" s="55">
+        <f>E29+(E31+E30)*E36</f>
+        <v/>
+      </c>
+      <c r="F39" s="55">
+        <f>F29+(F31+F30)*F36</f>
+        <v/>
+      </c>
+      <c r="G39" s="55">
+        <f>G29+(G31+G30)*G36</f>
+        <v/>
+      </c>
+      <c r="H39" s="55">
+        <f>H29+(H31+H30)*H36</f>
+        <v/>
+      </c>
+      <c r="I39" s="55">
+        <f>I29+(I31+I30)*I36</f>
+        <v/>
+      </c>
+      <c r="J39" s="55">
+        <f>J29+(J31+J30)*J36</f>
+        <v/>
+      </c>
+      <c r="K39" s="55">
+        <f>K29+(K31+K30)*K36</f>
+        <v/>
+      </c>
+      <c r="L39" s="55">
+        <f>L29+(L31+L30)*L36</f>
+        <v/>
+      </c>
+      <c r="M39" s="55">
+        <f>M29+(M31+M30)*M36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="20" t="inlineStr">
+        <is>
+          <t>Salesperson throughput</t>
+        </is>
+      </c>
+      <c r="B40" s="21" t="n"/>
+      <c r="D40" s="21" t="n"/>
+      <c r="E40" s="21" t="n"/>
+      <c r="F40" s="21" t="n"/>
+      <c r="G40" s="21" t="n"/>
+      <c r="H40" s="21" t="n"/>
+      <c r="I40" s="21" t="n"/>
+      <c r="J40" s="21" t="n"/>
+      <c r="K40" s="21" t="n"/>
+      <c r="L40" s="21" t="n"/>
+      <c r="M40" s="21" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="7" t="inlineStr">
+        <is>
+          <t>Opportunities a salesperson can manage</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 × change</t>
+        </is>
+      </c>
+      <c r="D41" s="55">
+        <f>v_opportunities_capacity*(1+D15)</f>
+        <v/>
+      </c>
+      <c r="E41" s="55">
+        <f>v_opportunities_capacity*(1+E15)</f>
+        <v/>
+      </c>
+      <c r="F41" s="55">
+        <f>v_opportunities_capacity*(1+F15)</f>
+        <v/>
+      </c>
+      <c r="G41" s="55">
+        <f>v_opportunities_capacity*(1+G15)</f>
+        <v/>
+      </c>
+      <c r="H41" s="55">
+        <f>v_opportunities_capacity*(1+H15)</f>
+        <v/>
+      </c>
+      <c r="I41" s="55">
+        <f>v_opportunities_capacity*(1+I15)</f>
+        <v/>
+      </c>
+      <c r="J41" s="55">
+        <f>v_opportunities_capacity*(1+J15)</f>
+        <v/>
+      </c>
+      <c r="K41" s="55">
+        <f>v_opportunities_capacity*(1+K15)</f>
+        <v/>
+      </c>
+      <c r="L41" s="55">
+        <f>v_opportunities_capacity*(1+L15)</f>
+        <v/>
+      </c>
+      <c r="M41" s="55">
+        <f>v_opportunities_capacity*(1+M15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="7" t="inlineStr">
+        <is>
+          <t>Opportunities each salesperson holds</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 pipeline data × change (blank if not provided)</t>
+        </is>
+      </c>
+      <c r="D42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+D16))</f>
+        <v/>
+      </c>
+      <c r="E42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+E16))</f>
+        <v/>
+      </c>
+      <c r="F42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+F16))</f>
+        <v/>
+      </c>
+      <c r="G42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+G16))</f>
+        <v/>
+      </c>
+      <c r="H42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+H16))</f>
+        <v/>
+      </c>
+      <c r="I42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+I16))</f>
+        <v/>
+      </c>
+      <c r="J42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+J16))</f>
+        <v/>
+      </c>
+      <c r="K42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+K16))</f>
+        <v/>
+      </c>
+      <c r="L42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+L16))</f>
+        <v/>
+      </c>
+      <c r="M42" s="55">
+        <f>IF(N(v_opportunities_load)=0,"",v_opportunities_load*(1+M16))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>Opportunities worked at once</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>The lower of what they hold and what they can manage</t>
+        </is>
+      </c>
+      <c r="D43" s="55">
+        <f>IF(D42="",D41,MIN(D42,D41))</f>
+        <v/>
+      </c>
+      <c r="E43" s="55">
+        <f>IF(E42="",E41,MIN(E42,E41))</f>
+        <v/>
+      </c>
+      <c r="F43" s="55">
+        <f>IF(F42="",F41,MIN(F42,F41))</f>
+        <v/>
+      </c>
+      <c r="G43" s="55">
+        <f>IF(G42="",G41,MIN(G42,G41))</f>
+        <v/>
+      </c>
+      <c r="H43" s="55">
+        <f>IF(H42="",H41,MIN(H42,H41))</f>
+        <v/>
+      </c>
+      <c r="I43" s="55">
+        <f>IF(I42="",I41,MIN(I42,I41))</f>
+        <v/>
+      </c>
+      <c r="J43" s="55">
+        <f>IF(J42="",J41,MIN(J42,J41))</f>
+        <v/>
+      </c>
+      <c r="K43" s="55">
+        <f>IF(K42="",K41,MIN(K42,K41))</f>
+        <v/>
+      </c>
+      <c r="L43" s="55">
+        <f>IF(L42="",L41,MIN(L42,L41))</f>
+        <v/>
+      </c>
+      <c r="M43" s="55">
+        <f>IF(M42="",M41,MIN(M42,M41))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="7" t="inlineStr">
+        <is>
+          <t>Utilization of capacity</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>Held ÷ can manage</t>
+        </is>
+      </c>
+      <c r="D44" s="57">
+        <f>IF(D42="","",D42/D41)</f>
+        <v/>
+      </c>
+      <c r="E44" s="57">
+        <f>IF(E42="","",E42/E41)</f>
+        <v/>
+      </c>
+      <c r="F44" s="57">
+        <f>IF(F42="","",F42/F41)</f>
+        <v/>
+      </c>
+      <c r="G44" s="57">
+        <f>IF(G42="","",G42/G41)</f>
+        <v/>
+      </c>
+      <c r="H44" s="57">
+        <f>IF(H42="","",H42/H41)</f>
+        <v/>
+      </c>
+      <c r="I44" s="57">
+        <f>IF(I42="","",I42/I41)</f>
+        <v/>
+      </c>
+      <c r="J44" s="57">
+        <f>IF(J42="","",J42/J41)</f>
+        <v/>
+      </c>
+      <c r="K44" s="57">
+        <f>IF(K42="","",K42/K41)</f>
+        <v/>
+      </c>
+      <c r="L44" s="57">
+        <f>IF(L42="","",L42/L41)</f>
+        <v/>
+      </c>
+      <c r="M44" s="57">
+        <f>IF(M42="","",M42/M41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="7" t="inlineStr">
+        <is>
+          <t>Sales cycle (months)</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 × change</t>
+        </is>
+      </c>
+      <c r="D45" s="56">
+        <f>v_cycle_months*(1+D17)</f>
+        <v/>
+      </c>
+      <c r="E45" s="56">
+        <f>v_cycle_months*(1+E17)</f>
+        <v/>
+      </c>
+      <c r="F45" s="56">
+        <f>v_cycle_months*(1+F17)</f>
+        <v/>
+      </c>
+      <c r="G45" s="56">
+        <f>v_cycle_months*(1+G17)</f>
+        <v/>
+      </c>
+      <c r="H45" s="56">
+        <f>v_cycle_months*(1+H17)</f>
+        <v/>
+      </c>
+      <c r="I45" s="56">
+        <f>v_cycle_months*(1+I17)</f>
+        <v/>
+      </c>
+      <c r="J45" s="56">
+        <f>v_cycle_months*(1+J17)</f>
+        <v/>
+      </c>
+      <c r="K45" s="56">
+        <f>v_cycle_months*(1+K17)</f>
+        <v/>
+      </c>
+      <c r="L45" s="56">
+        <f>v_cycle_months*(1+L17)</f>
+        <v/>
+      </c>
+      <c r="M45" s="56">
+        <f>v_cycle_months*(1+M17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="7" t="inlineStr">
+        <is>
+          <t>Opportunities resolved per salesperson per year</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>Little's Law: worked × 12 ÷ cycle</t>
+        </is>
+      </c>
+      <c r="D46" s="55">
+        <f>D43*12/D45</f>
+        <v/>
+      </c>
+      <c r="E46" s="55">
+        <f>E43*12/E45</f>
+        <v/>
+      </c>
+      <c r="F46" s="55">
+        <f>F43*12/F45</f>
+        <v/>
+      </c>
+      <c r="G46" s="55">
+        <f>G43*12/G45</f>
+        <v/>
+      </c>
+      <c r="H46" s="55">
+        <f>H43*12/H45</f>
+        <v/>
+      </c>
+      <c r="I46" s="55">
+        <f>I43*12/I45</f>
+        <v/>
+      </c>
+      <c r="J46" s="55">
+        <f>J43*12/J45</f>
+        <v/>
+      </c>
+      <c r="K46" s="55">
+        <f>K43*12/K45</f>
+        <v/>
+      </c>
+      <c r="L46" s="55">
+        <f>L43*12/L45</f>
+        <v/>
+      </c>
+      <c r="M46" s="55">
+        <f>M43*12/M45</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="inlineStr">
+        <is>
+          <t>Close rate</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 × change</t>
+        </is>
+      </c>
+      <c r="D47" s="58">
+        <f>v_win_rate*(1+D18)</f>
+        <v/>
+      </c>
+      <c r="E47" s="58">
+        <f>v_win_rate*(1+E18)</f>
+        <v/>
+      </c>
+      <c r="F47" s="58">
+        <f>v_win_rate*(1+F18)</f>
+        <v/>
+      </c>
+      <c r="G47" s="58">
+        <f>v_win_rate*(1+G18)</f>
+        <v/>
+      </c>
+      <c r="H47" s="58">
+        <f>v_win_rate*(1+H18)</f>
+        <v/>
+      </c>
+      <c r="I47" s="58">
+        <f>v_win_rate*(1+I18)</f>
+        <v/>
+      </c>
+      <c r="J47" s="58">
+        <f>v_win_rate*(1+J18)</f>
+        <v/>
+      </c>
+      <c r="K47" s="58">
+        <f>v_win_rate*(1+K18)</f>
+        <v/>
+      </c>
+      <c r="L47" s="58">
+        <f>v_win_rate*(1+L18)</f>
+        <v/>
+      </c>
+      <c r="M47" s="58">
+        <f>v_win_rate*(1+M18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>Contracts per productive territory</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>Resolved × close rate</t>
+        </is>
+      </c>
+      <c r="D48" s="55">
+        <f>D46*D47</f>
+        <v/>
+      </c>
+      <c r="E48" s="55">
+        <f>E46*E47</f>
+        <v/>
+      </c>
+      <c r="F48" s="55">
+        <f>F46*F47</f>
+        <v/>
+      </c>
+      <c r="G48" s="55">
+        <f>G46*G47</f>
+        <v/>
+      </c>
+      <c r="H48" s="55">
+        <f>H46*H47</f>
+        <v/>
+      </c>
+      <c r="I48" s="55">
+        <f>I46*I47</f>
+        <v/>
+      </c>
+      <c r="J48" s="55">
+        <f>J46*J47</f>
+        <v/>
+      </c>
+      <c r="K48" s="55">
+        <f>K46*K47</f>
+        <v/>
+      </c>
+      <c r="L48" s="55">
+        <f>L46*L47</f>
+        <v/>
+      </c>
+      <c r="M48" s="55">
+        <f>M46*M47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="7" t="inlineStr">
+        <is>
+          <t>Average revenue per contract</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 × change</t>
+        </is>
+      </c>
+      <c r="D49" s="59">
+        <f>v_deal_size*(1+D19)</f>
+        <v/>
+      </c>
+      <c r="E49" s="59">
+        <f>v_deal_size*(1+E19)</f>
+        <v/>
+      </c>
+      <c r="F49" s="59">
+        <f>v_deal_size*(1+F19)</f>
+        <v/>
+      </c>
+      <c r="G49" s="59">
+        <f>v_deal_size*(1+G19)</f>
+        <v/>
+      </c>
+      <c r="H49" s="59">
+        <f>v_deal_size*(1+H19)</f>
+        <v/>
+      </c>
+      <c r="I49" s="59">
+        <f>v_deal_size*(1+I19)</f>
+        <v/>
+      </c>
+      <c r="J49" s="59">
+        <f>v_deal_size*(1+J19)</f>
+        <v/>
+      </c>
+      <c r="K49" s="59">
+        <f>v_deal_size*(1+K19)</f>
+        <v/>
+      </c>
+      <c r="L49" s="59">
+        <f>v_deal_size*(1+L19)</f>
+        <v/>
+      </c>
+      <c r="M49" s="59">
+        <f>v_deal_size*(1+M19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>Revenue per productive territory</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>Contracts × revenue per contract</t>
+        </is>
+      </c>
+      <c r="D50" s="59">
+        <f>D48*D49</f>
+        <v/>
+      </c>
+      <c r="E50" s="59">
+        <f>E48*E49</f>
+        <v/>
+      </c>
+      <c r="F50" s="59">
+        <f>F48*F49</f>
+        <v/>
+      </c>
+      <c r="G50" s="59">
+        <f>G48*G49</f>
+        <v/>
+      </c>
+      <c r="H50" s="59">
+        <f>H48*H49</f>
+        <v/>
+      </c>
+      <c r="I50" s="59">
+        <f>I48*I49</f>
+        <v/>
+      </c>
+      <c r="J50" s="59">
+        <f>J48*J49</f>
+        <v/>
+      </c>
+      <c r="K50" s="59">
+        <f>K48*K49</f>
+        <v/>
+      </c>
+      <c r="L50" s="59">
+        <f>L48*L49</f>
+        <v/>
+      </c>
+      <c r="M50" s="59">
+        <f>M48*M49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="20" t="inlineStr">
+        <is>
+          <t>Income statement</t>
+        </is>
+      </c>
+      <c r="B51" s="21" t="n"/>
+      <c r="D51" s="21" t="n"/>
+      <c r="E51" s="21" t="n"/>
+      <c r="F51" s="21" t="n"/>
+      <c r="G51" s="21" t="n"/>
+      <c r="H51" s="21" t="n"/>
+      <c r="I51" s="21" t="n"/>
+      <c r="J51" s="21" t="n"/>
+      <c r="K51" s="21" t="n"/>
+      <c r="L51" s="21" t="n"/>
+      <c r="M51" s="21" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>Contracts</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>Per territory × productive territory-years</t>
+        </is>
+      </c>
+      <c r="D52" s="60">
+        <f>D48*D38</f>
+        <v/>
+      </c>
+      <c r="E52" s="60">
+        <f>E48*E38</f>
+        <v/>
+      </c>
+      <c r="F52" s="60">
+        <f>F48*F38</f>
+        <v/>
+      </c>
+      <c r="G52" s="60">
+        <f>G48*G38</f>
+        <v/>
+      </c>
+      <c r="H52" s="60">
+        <f>H48*H38</f>
+        <v/>
+      </c>
+      <c r="I52" s="60">
+        <f>I48*I38</f>
+        <v/>
+      </c>
+      <c r="J52" s="60">
+        <f>J48*J38</f>
+        <v/>
+      </c>
+      <c r="K52" s="60">
+        <f>K48*K38</f>
+        <v/>
+      </c>
+      <c r="L52" s="60">
+        <f>L48*L38</f>
+        <v/>
+      </c>
+      <c r="M52" s="60">
+        <f>M48*M38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>Per territory × productive territory-years</t>
+        </is>
+      </c>
+      <c r="D53" s="61">
+        <f>D50*D38</f>
+        <v/>
+      </c>
+      <c r="E53" s="61">
+        <f>E50*E38</f>
+        <v/>
+      </c>
+      <c r="F53" s="61">
+        <f>F50*F38</f>
+        <v/>
+      </c>
+      <c r="G53" s="61">
+        <f>G50*G38</f>
+        <v/>
+      </c>
+      <c r="H53" s="61">
+        <f>H50*H38</f>
+        <v/>
+      </c>
+      <c r="I53" s="61">
+        <f>I50*I38</f>
+        <v/>
+      </c>
+      <c r="J53" s="61">
+        <f>J50*J38</f>
+        <v/>
+      </c>
+      <c r="K53" s="61">
+        <f>K50*K38</f>
+        <v/>
+      </c>
+      <c r="L53" s="61">
+        <f>L50*L38</f>
+        <v/>
+      </c>
+      <c r="M53" s="61">
+        <f>M50*M38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>Cost of revenue</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>Revenue × tab 1 %</t>
+        </is>
+      </c>
+      <c r="D54" s="59">
+        <f>D53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+      <c r="E54" s="59">
+        <f>E53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+      <c r="F54" s="59">
+        <f>F53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+      <c r="G54" s="59">
+        <f>G53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+      <c r="H54" s="59">
+        <f>H53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+      <c r="I54" s="59">
+        <f>I53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+      <c r="J54" s="59">
+        <f>J53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+      <c r="K54" s="59">
+        <f>K53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+      <c r="L54" s="59">
+        <f>L53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+      <c r="M54" s="59">
+        <f>M53*v_cost_of_revenue_pct</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="7" t="inlineStr">
+        <is>
+          <t>Research and development</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>Revenue × tab 1 %</t>
+        </is>
+      </c>
+      <c r="D55" s="59">
+        <f>D53*v_rnd_pct</f>
+        <v/>
+      </c>
+      <c r="E55" s="59">
+        <f>E53*v_rnd_pct</f>
+        <v/>
+      </c>
+      <c r="F55" s="59">
+        <f>F53*v_rnd_pct</f>
+        <v/>
+      </c>
+      <c r="G55" s="59">
+        <f>G53*v_rnd_pct</f>
+        <v/>
+      </c>
+      <c r="H55" s="59">
+        <f>H53*v_rnd_pct</f>
+        <v/>
+      </c>
+      <c r="I55" s="59">
+        <f>I53*v_rnd_pct</f>
+        <v/>
+      </c>
+      <c r="J55" s="59">
+        <f>J53*v_rnd_pct</f>
+        <v/>
+      </c>
+      <c r="K55" s="59">
+        <f>K53*v_rnd_pct</f>
+        <v/>
+      </c>
+      <c r="L55" s="59">
+        <f>L53*v_rnd_pct</f>
+        <v/>
+      </c>
+      <c r="M55" s="59">
+        <f>M53*v_rnd_pct</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>General and administrative</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>Revenue × tab 1 %</t>
+        </is>
+      </c>
+      <c r="D56" s="59">
+        <f>D53*v_gna_pct</f>
+        <v/>
+      </c>
+      <c r="E56" s="59">
+        <f>E53*v_gna_pct</f>
+        <v/>
+      </c>
+      <c r="F56" s="59">
+        <f>F53*v_gna_pct</f>
+        <v/>
+      </c>
+      <c r="G56" s="59">
+        <f>G53*v_gna_pct</f>
+        <v/>
+      </c>
+      <c r="H56" s="59">
+        <f>H53*v_gna_pct</f>
+        <v/>
+      </c>
+      <c r="I56" s="59">
+        <f>I53*v_gna_pct</f>
+        <v/>
+      </c>
+      <c r="J56" s="59">
+        <f>J53*v_gna_pct</f>
+        <v/>
+      </c>
+      <c r="K56" s="59">
+        <f>K53*v_gna_pct</f>
+        <v/>
+      </c>
+      <c r="L56" s="59">
+        <f>L53*v_gna_pct</f>
+        <v/>
+      </c>
+      <c r="M56" s="59">
+        <f>M53*v_gna_pct</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="7" t="inlineStr">
+        <is>
+          <t>Salesperson salaries, load and travel</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>(Loaded salary + travel) × salesperson-years paid</t>
+        </is>
+      </c>
+      <c r="D57" s="59">
+        <f>(v_loaded_salary*(1+D20)+v_travel_per_salesperson)*D39</f>
+        <v/>
+      </c>
+      <c r="E57" s="59">
+        <f>(v_loaded_salary*(1+E20)+v_travel_per_salesperson)*E39</f>
+        <v/>
+      </c>
+      <c r="F57" s="59">
+        <f>(v_loaded_salary*(1+F20)+v_travel_per_salesperson)*F39</f>
+        <v/>
+      </c>
+      <c r="G57" s="59">
+        <f>(v_loaded_salary*(1+G20)+v_travel_per_salesperson)*G39</f>
+        <v/>
+      </c>
+      <c r="H57" s="59">
+        <f>(v_loaded_salary*(1+H20)+v_travel_per_salesperson)*H39</f>
+        <v/>
+      </c>
+      <c r="I57" s="59">
+        <f>(v_loaded_salary*(1+I20)+v_travel_per_salesperson)*I39</f>
+        <v/>
+      </c>
+      <c r="J57" s="59">
+        <f>(v_loaded_salary*(1+J20)+v_travel_per_salesperson)*J39</f>
+        <v/>
+      </c>
+      <c r="K57" s="59">
+        <f>(v_loaded_salary*(1+K20)+v_travel_per_salesperson)*K39</f>
+        <v/>
+      </c>
+      <c r="L57" s="59">
+        <f>(v_loaded_salary*(1+L20)+v_travel_per_salesperson)*L39</f>
+        <v/>
+      </c>
+      <c r="M57" s="59">
+        <f>(v_loaded_salary*(1+M20)+v_travel_per_salesperson)*M39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>Commissions</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>Rate × revenue (only on revenue produced)</t>
+        </is>
+      </c>
+      <c r="D58" s="59">
+        <f>v_commission_rate*(1+D21)*D53</f>
+        <v/>
+      </c>
+      <c r="E58" s="59">
+        <f>v_commission_rate*(1+E21)*E53</f>
+        <v/>
+      </c>
+      <c r="F58" s="59">
+        <f>v_commission_rate*(1+F21)*F53</f>
+        <v/>
+      </c>
+      <c r="G58" s="59">
+        <f>v_commission_rate*(1+G21)*G53</f>
+        <v/>
+      </c>
+      <c r="H58" s="59">
+        <f>v_commission_rate*(1+H21)*H53</f>
+        <v/>
+      </c>
+      <c r="I58" s="59">
+        <f>v_commission_rate*(1+I21)*I53</f>
+        <v/>
+      </c>
+      <c r="J58" s="59">
+        <f>v_commission_rate*(1+J21)*J53</f>
+        <v/>
+      </c>
+      <c r="K58" s="59">
+        <f>v_commission_rate*(1+K21)*K53</f>
+        <v/>
+      </c>
+      <c r="L58" s="59">
+        <f>v_commission_rate*(1+L21)*L53</f>
+        <v/>
+      </c>
+      <c r="M58" s="59">
+        <f>v_commission_rate*(1+M21)*M53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="7" t="inlineStr">
+        <is>
+          <t>Sales overhead</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 + change</t>
+        </is>
+      </c>
+      <c r="D59" s="59">
+        <f>v_sales_overhead+D22</f>
+        <v/>
+      </c>
+      <c r="E59" s="59">
+        <f>v_sales_overhead+E22</f>
+        <v/>
+      </c>
+      <c r="F59" s="59">
+        <f>v_sales_overhead+F22</f>
+        <v/>
+      </c>
+      <c r="G59" s="59">
+        <f>v_sales_overhead+G22</f>
+        <v/>
+      </c>
+      <c r="H59" s="59">
+        <f>v_sales_overhead+H22</f>
+        <v/>
+      </c>
+      <c r="I59" s="59">
+        <f>v_sales_overhead+I22</f>
+        <v/>
+      </c>
+      <c r="J59" s="59">
+        <f>v_sales_overhead+J22</f>
+        <v/>
+      </c>
+      <c r="K59" s="59">
+        <f>v_sales_overhead+K22</f>
+        <v/>
+      </c>
+      <c r="L59" s="59">
+        <f>v_sales_overhead+L22</f>
+        <v/>
+      </c>
+      <c r="M59" s="59">
+        <f>v_sales_overhead+M22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>Marketing</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>Tab 1 + change</t>
+        </is>
+      </c>
+      <c r="D60" s="59">
+        <f>v_marketing+D23</f>
+        <v/>
+      </c>
+      <c r="E60" s="59">
+        <f>v_marketing+E23</f>
+        <v/>
+      </c>
+      <c r="F60" s="59">
+        <f>v_marketing+F23</f>
+        <v/>
+      </c>
+      <c r="G60" s="59">
+        <f>v_marketing+G23</f>
+        <v/>
+      </c>
+      <c r="H60" s="59">
+        <f>v_marketing+H23</f>
+        <v/>
+      </c>
+      <c r="I60" s="59">
+        <f>v_marketing+I23</f>
+        <v/>
+      </c>
+      <c r="J60" s="59">
+        <f>v_marketing+J23</f>
+        <v/>
+      </c>
+      <c r="K60" s="59">
+        <f>v_marketing+K23</f>
+        <v/>
+      </c>
+      <c r="L60" s="59">
+        <f>v_marketing+L23</f>
+        <v/>
+      </c>
+      <c r="M60" s="59">
+        <f>v_marketing+M23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="7" t="inlineStr">
+        <is>
+          <t>Cost of making the change</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>From the change rows</t>
+        </is>
+      </c>
+      <c r="D61" s="59">
+        <f>D24</f>
+        <v/>
+      </c>
+      <c r="E61" s="59">
+        <f>E24</f>
+        <v/>
+      </c>
+      <c r="F61" s="59">
+        <f>F24</f>
+        <v/>
+      </c>
+      <c r="G61" s="59">
+        <f>G24</f>
+        <v/>
+      </c>
+      <c r="H61" s="59">
+        <f>H24</f>
+        <v/>
+      </c>
+      <c r="I61" s="59">
+        <f>I24</f>
+        <v/>
+      </c>
+      <c r="J61" s="59">
+        <f>J24</f>
+        <v/>
+      </c>
+      <c r="K61" s="59">
+        <f>K24</f>
+        <v/>
+      </c>
+      <c r="L61" s="59">
+        <f>L24</f>
+        <v/>
+      </c>
+      <c r="M61" s="59">
+        <f>M24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>Total costs</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>Sum of the lines above</t>
+        </is>
+      </c>
+      <c r="D62" s="59">
+        <f>D54+D55+D56+D57+D58+D59+D60+D61</f>
+        <v/>
+      </c>
+      <c r="E62" s="59">
+        <f>E54+E55+E56+E57+E58+E59+E60+E61</f>
+        <v/>
+      </c>
+      <c r="F62" s="59">
+        <f>F54+F55+F56+F57+F58+F59+F60+F61</f>
+        <v/>
+      </c>
+      <c r="G62" s="59">
+        <f>G54+G55+G56+G57+G58+G59+G60+G61</f>
+        <v/>
+      </c>
+      <c r="H62" s="59">
+        <f>H54+H55+H56+H57+H58+H59+H60+H61</f>
+        <v/>
+      </c>
+      <c r="I62" s="59">
+        <f>I54+I55+I56+I57+I58+I59+I60+I61</f>
+        <v/>
+      </c>
+      <c r="J62" s="59">
+        <f>J54+J55+J56+J57+J58+J59+J60+J61</f>
+        <v/>
+      </c>
+      <c r="K62" s="59">
+        <f>K54+K55+K56+K57+K58+K59+K60+K61</f>
+        <v/>
+      </c>
+      <c r="L62" s="59">
+        <f>L54+L55+L56+L57+L58+L59+L60+L61</f>
+        <v/>
+      </c>
+      <c r="M62" s="59">
+        <f>M54+M55+M56+M57+M58+M59+M60+M61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>Operating income</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>Revenue − total costs</t>
+        </is>
+      </c>
+      <c r="D63" s="61">
+        <f>D53-D62</f>
+        <v/>
+      </c>
+      <c r="E63" s="61">
+        <f>E53-E62</f>
+        <v/>
+      </c>
+      <c r="F63" s="61">
+        <f>F53-F62</f>
+        <v/>
+      </c>
+      <c r="G63" s="61">
+        <f>G53-G62</f>
+        <v/>
+      </c>
+      <c r="H63" s="61">
+        <f>H53-H62</f>
+        <v/>
+      </c>
+      <c r="I63" s="61">
+        <f>I53-I62</f>
+        <v/>
+      </c>
+      <c r="J63" s="61">
+        <f>J53-J62</f>
+        <v/>
+      </c>
+      <c r="K63" s="61">
+        <f>K53-K62</f>
+        <v/>
+      </c>
+      <c r="L63" s="61">
+        <f>L53-L62</f>
+        <v/>
+      </c>
+      <c r="M63" s="61">
+        <f>M53-M62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>Operating margin</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>Operating income ÷ revenue</t>
+        </is>
+      </c>
+      <c r="D64" s="58">
+        <f>IFERROR(D63/D53,"")</f>
+        <v/>
+      </c>
+      <c r="E64" s="58">
+        <f>IFERROR(E63/E53,"")</f>
+        <v/>
+      </c>
+      <c r="F64" s="58">
+        <f>IFERROR(F63/F53,"")</f>
+        <v/>
+      </c>
+      <c r="G64" s="58">
+        <f>IFERROR(G63/G53,"")</f>
+        <v/>
+      </c>
+      <c r="H64" s="58">
+        <f>IFERROR(H63/H53,"")</f>
+        <v/>
+      </c>
+      <c r="I64" s="58">
+        <f>IFERROR(I63/I53,"")</f>
+        <v/>
+      </c>
+      <c r="J64" s="58">
+        <f>IFERROR(J63/J53,"")</f>
+        <v/>
+      </c>
+      <c r="K64" s="58">
+        <f>IFERROR(K63/K53,"")</f>
+        <v/>
+      </c>
+      <c r="L64" s="58">
+        <f>IFERROR(L63/L53,"")</f>
+        <v/>
+      </c>
+      <c r="M64" s="58">
+        <f>IFERROR(M63/M53,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="20" t="inlineStr">
+        <is>
+          <t>Change from baseline and true-up</t>
+        </is>
+      </c>
+      <c r="B65" s="21" t="n"/>
+      <c r="D65" s="21" t="n"/>
+      <c r="E65" s="21" t="n"/>
+      <c r="F65" s="21" t="n"/>
+      <c r="G65" s="21" t="n"/>
+      <c r="H65" s="21" t="n"/>
+      <c r="I65" s="21" t="n"/>
+      <c r="J65" s="21" t="n"/>
+      <c r="K65" s="21" t="n"/>
+      <c r="L65" s="21" t="n"/>
+      <c r="M65" s="21" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>Change in revenue</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr"/>
+      <c r="D66" s="59" t="n"/>
+      <c r="E66" s="59">
+        <f>E53-$D$53</f>
+        <v/>
+      </c>
+      <c r="F66" s="59">
+        <f>F53-$D$53</f>
+        <v/>
+      </c>
+      <c r="G66" s="59">
+        <f>G53-$D$53</f>
+        <v/>
+      </c>
+      <c r="H66" s="59">
+        <f>H53-$D$53</f>
+        <v/>
+      </c>
+      <c r="I66" s="59">
+        <f>I53-$D$53</f>
+        <v/>
+      </c>
+      <c r="J66" s="59">
+        <f>J53-$D$53</f>
+        <v/>
+      </c>
+      <c r="K66" s="59">
+        <f>K53-$D$53</f>
+        <v/>
+      </c>
+      <c r="L66" s="59">
+        <f>L53-$D$53</f>
+        <v/>
+      </c>
+      <c r="M66" s="59">
+        <f>M53-$D$53</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>Change in total costs</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr"/>
+      <c r="D67" s="59" t="n"/>
+      <c r="E67" s="59">
+        <f>E62-$D$62</f>
+        <v/>
+      </c>
+      <c r="F67" s="59">
+        <f>F62-$D$62</f>
+        <v/>
+      </c>
+      <c r="G67" s="59">
+        <f>G62-$D$62</f>
+        <v/>
+      </c>
+      <c r="H67" s="59">
+        <f>H62-$D$62</f>
+        <v/>
+      </c>
+      <c r="I67" s="59">
+        <f>I62-$D$62</f>
+        <v/>
+      </c>
+      <c r="J67" s="59">
+        <f>J62-$D$62</f>
+        <v/>
+      </c>
+      <c r="K67" s="59">
+        <f>K62-$D$62</f>
+        <v/>
+      </c>
+      <c r="L67" s="59">
+        <f>L62-$D$62</f>
+        <v/>
+      </c>
+      <c r="M67" s="59">
+        <f>M62-$D$62</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>Change in operating income</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr"/>
+      <c r="D68" s="61" t="n"/>
+      <c r="E68" s="61">
+        <f>E63-$D$63</f>
+        <v/>
+      </c>
+      <c r="F68" s="61">
+        <f>F63-$D$63</f>
+        <v/>
+      </c>
+      <c r="G68" s="61">
+        <f>G63-$D$63</f>
+        <v/>
+      </c>
+      <c r="H68" s="61">
+        <f>H63-$D$63</f>
+        <v/>
+      </c>
+      <c r="I68" s="61">
+        <f>I63-$D$63</f>
+        <v/>
+      </c>
+      <c r="J68" s="61">
+        <f>J63-$D$63</f>
+        <v/>
+      </c>
+      <c r="K68" s="61">
+        <f>K63-$D$63</f>
+        <v/>
+      </c>
+      <c r="L68" s="61">
+        <f>L63-$D$63</f>
+        <v/>
+      </c>
+      <c r="M68" s="61">
+        <f>M63-$D$63</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>Change in operating income, %</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr"/>
+      <c r="D69" s="62" t="n"/>
+      <c r="E69" s="62">
+        <f>IFERROR(E68/ABS($D$63),"")</f>
+        <v/>
+      </c>
+      <c r="F69" s="62">
+        <f>IFERROR(F68/ABS($D$63),"")</f>
+        <v/>
+      </c>
+      <c r="G69" s="62">
+        <f>IFERROR(G68/ABS($D$63),"")</f>
+        <v/>
+      </c>
+      <c r="H69" s="62">
+        <f>IFERROR(H68/ABS($D$63),"")</f>
+        <v/>
+      </c>
+      <c r="I69" s="62">
+        <f>IFERROR(I68/ABS($D$63),"")</f>
+        <v/>
+      </c>
+      <c r="J69" s="62">
+        <f>IFERROR(J68/ABS($D$63),"")</f>
+        <v/>
+      </c>
+      <c r="K69" s="62">
+        <f>IFERROR(K68/ABS($D$63),"")</f>
+        <v/>
+      </c>
+      <c r="L69" s="62">
+        <f>IFERROR(L68/ABS($D$63),"")</f>
+        <v/>
+      </c>
+      <c r="M69" s="62">
+        <f>IFERROR(M68/ABS($D$63),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>Unexplained difference (must be 0)</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>Change in revenue − change in costs − change in operating income</t>
+        </is>
+      </c>
+      <c r="D70" s="59">
+        <f>D66-D67-D68</f>
+        <v/>
+      </c>
+      <c r="E70" s="59">
+        <f>E66-E67-E68</f>
+        <v/>
+      </c>
+      <c r="F70" s="59">
+        <f>F66-F67-F68</f>
+        <v/>
+      </c>
+      <c r="G70" s="59">
+        <f>G66-G67-G68</f>
+        <v/>
+      </c>
+      <c r="H70" s="59">
+        <f>H66-H67-H68</f>
+        <v/>
+      </c>
+      <c r="I70" s="59">
+        <f>I66-I67-I68</f>
+        <v/>
+      </c>
+      <c r="J70" s="59">
+        <f>J66-J67-J68</f>
+        <v/>
+      </c>
+      <c r="K70" s="59">
+        <f>K66-K67-K68</f>
+        <v/>
+      </c>
+      <c r="L70" s="59">
+        <f>L66-L67-L68</f>
+        <v/>
+      </c>
+      <c r="M70" s="59">
+        <f>M66-M67-M68</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>True-up</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>Every change in profit is explained by a change in revenue or cost</t>
+        </is>
+      </c>
+      <c r="D71" s="63">
+        <f>IF(ABS(D70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+      <c r="E71" s="63">
+        <f>IF(ABS(E70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+      <c r="F71" s="63">
+        <f>IF(ABS(F70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+      <c r="G71" s="63">
+        <f>IF(ABS(G70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+      <c r="H71" s="63">
+        <f>IF(ABS(H70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+      <c r="I71" s="63">
+        <f>IF(ABS(I70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+      <c r="J71" s="63">
+        <f>IF(ABS(J70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+      <c r="K71" s="63">
+        <f>IF(ABS(K70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+      <c r="L71" s="63">
+        <f>IF(ABS(L70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+      <c r="M71" s="63">
+        <f>IF(ABS(M70)&lt;0.5,"Balanced","Check")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="20" t="inlineStr">
+        <is>
+          <t>Decision measures</t>
+        </is>
+      </c>
+      <c r="B72" s="21" t="n"/>
+      <c r="D72" s="21" t="n"/>
+      <c r="E72" s="21" t="n"/>
+      <c r="F72" s="21" t="n"/>
+      <c r="G72" s="21" t="n"/>
+      <c r="H72" s="21" t="n"/>
+      <c r="I72" s="21" t="n"/>
+      <c r="J72" s="21" t="n"/>
+      <c r="K72" s="21" t="n"/>
+      <c r="L72" s="21" t="n"/>
+      <c r="M72" s="21" t="n"/>
+    </row>
+    <row r="73" ht="28" customHeight="1">
+      <c r="A73" s="4" t="inlineStr">
+        <is>
+          <t>Change in operating income before the cost of making the change</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr"/>
+      <c r="D73" s="59" t="n"/>
+      <c r="E73" s="59">
+        <f>E68+E61</f>
+        <v/>
+      </c>
+      <c r="F73" s="59">
+        <f>F68+F61</f>
+        <v/>
+      </c>
+      <c r="G73" s="59">
+        <f>G68+G61</f>
+        <v/>
+      </c>
+      <c r="H73" s="59">
+        <f>H68+H61</f>
+        <v/>
+      </c>
+      <c r="I73" s="59">
+        <f>I68+I61</f>
+        <v/>
+      </c>
+      <c r="J73" s="59">
+        <f>J68+J61</f>
+        <v/>
+      </c>
+      <c r="K73" s="59">
+        <f>K68+K61</f>
+        <v/>
+      </c>
+      <c r="L73" s="59">
+        <f>L68+L61</f>
+        <v/>
+      </c>
+      <c r="M73" s="59">
+        <f>M68+M61</f>
+        <v/>
+      </c>
+    </row>
+    <row r="74" ht="28" customHeight="1">
+      <c r="A74" s="64" t="inlineStr">
+        <is>
+          <t>Most you could spend on this change and still match the comparison scenario</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>This scenario's gain before its cost − the comparison scenario's gain</t>
+        </is>
+      </c>
+      <c r="D74" s="61" t="n"/>
+      <c r="E74" s="61">
+        <f>E73-INDEX($D$73:$M$73,MATCH(wi_compare,$D$7:$M$7,0))</f>
+        <v/>
+      </c>
+      <c r="F74" s="61">
+        <f>F73-INDEX($D$73:$M$73,MATCH(wi_compare,$D$7:$M$7,0))</f>
+        <v/>
+      </c>
+      <c r="G74" s="61">
+        <f>G73-INDEX($D$73:$M$73,MATCH(wi_compare,$D$7:$M$7,0))</f>
+        <v/>
+      </c>
+      <c r="H74" s="61">
+        <f>H73-INDEX($D$73:$M$73,MATCH(wi_compare,$D$7:$M$7,0))</f>
+        <v/>
+      </c>
+      <c r="I74" s="61">
+        <f>I73-INDEX($D$73:$M$73,MATCH(wi_compare,$D$7:$M$7,0))</f>
+        <v/>
+      </c>
+      <c r="J74" s="61">
+        <f>J73-INDEX($D$73:$M$73,MATCH(wi_compare,$D$7:$M$7,0))</f>
+        <v/>
+      </c>
+      <c r="K74" s="61">
+        <f>K73-INDEX($D$73:$M$73,MATCH(wi_compare,$D$7:$M$7,0))</f>
+        <v/>
+      </c>
+      <c r="L74" s="61">
+        <f>L73-INDEX($D$73:$M$73,MATCH(wi_compare,$D$7:$M$7,0))</f>
+        <v/>
+      </c>
+      <c r="M74" s="61">
+        <f>M73-INDEX($D$73:$M$73,MATCH(wi_compare,$D$7:$M$7,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="7" t="inlineStr">
+        <is>
+          <t>Revenue per salesperson-year paid</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr"/>
+      <c r="D75" s="59">
+        <f>IFERROR(D53/D39,"")</f>
+        <v/>
+      </c>
+      <c r="E75" s="59">
+        <f>IFERROR(E53/E39,"")</f>
+        <v/>
+      </c>
+      <c r="F75" s="59">
+        <f>IFERROR(F53/F39,"")</f>
+        <v/>
+      </c>
+      <c r="G75" s="59">
+        <f>IFERROR(G53/G39,"")</f>
+        <v/>
+      </c>
+      <c r="H75" s="59">
+        <f>IFERROR(H53/H39,"")</f>
+        <v/>
+      </c>
+      <c r="I75" s="59">
+        <f>IFERROR(I53/I39,"")</f>
+        <v/>
+      </c>
+      <c r="J75" s="59">
+        <f>IFERROR(J53/J39,"")</f>
+        <v/>
+      </c>
+      <c r="K75" s="59">
+        <f>IFERROR(K53/K39,"")</f>
+        <v/>
+      </c>
+      <c r="L75" s="59">
+        <f>IFERROR(L53/L39,"")</f>
+        <v/>
+      </c>
+      <c r="M75" s="59">
+        <f>IFERROR(M53/M39,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="76" ht="66" customHeight="1">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>Guardrails</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>Flags results that leave known reality</t>
+        </is>
+      </c>
+      <c r="D76" s="63">
+        <f>IF(D47&gt;1,"Close rate above 100%: not possible",IF(D45&lt;=0,"Cycle must be above zero",IF(AND(D42&lt;&gt;"",D16&lt;&gt;0,D42&gt;D41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(D42&lt;&gt;"",D15&gt;0,D42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(D42="",D16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(D28=0,OR(D12&lt;&gt;0,_xlfn.ISFORMULA(D12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="E76" s="63">
+        <f>IF(E47&gt;1,"Close rate above 100%: not possible",IF(E45&lt;=0,"Cycle must be above zero",IF(AND(E42&lt;&gt;"",E16&lt;&gt;0,E42&gt;E41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(E42&lt;&gt;"",E15&gt;0,E42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(E42="",E16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(E28=0,OR(E12&lt;&gt;0,_xlfn.ISFORMULA(E12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="F76" s="63">
+        <f>IF(F47&gt;1,"Close rate above 100%: not possible",IF(F45&lt;=0,"Cycle must be above zero",IF(AND(F42&lt;&gt;"",F16&lt;&gt;0,F42&gt;F41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(F42&lt;&gt;"",F15&gt;0,F42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(F42="",F16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(F28=0,OR(F12&lt;&gt;0,_xlfn.ISFORMULA(F12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="G76" s="63">
+        <f>IF(G47&gt;1,"Close rate above 100%: not possible",IF(G45&lt;=0,"Cycle must be above zero",IF(AND(G42&lt;&gt;"",G16&lt;&gt;0,G42&gt;G41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(G42&lt;&gt;"",G15&gt;0,G42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(G42="",G16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(G28=0,OR(G12&lt;&gt;0,_xlfn.ISFORMULA(G12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="H76" s="63">
+        <f>IF(H47&gt;1,"Close rate above 100%: not possible",IF(H45&lt;=0,"Cycle must be above zero",IF(AND(H42&lt;&gt;"",H16&lt;&gt;0,H42&gt;H41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(H42&lt;&gt;"",H15&gt;0,H42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(H42="",H16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(H28=0,OR(H12&lt;&gt;0,_xlfn.ISFORMULA(H12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="I76" s="63">
+        <f>IF(I47&gt;1,"Close rate above 100%: not possible",IF(I45&lt;=0,"Cycle must be above zero",IF(AND(I42&lt;&gt;"",I16&lt;&gt;0,I42&gt;I41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(I42&lt;&gt;"",I15&gt;0,I42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(I42="",I16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(I28=0,OR(I12&lt;&gt;0,_xlfn.ISFORMULA(I12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="J76" s="63">
+        <f>IF(J47&gt;1,"Close rate above 100%: not possible",IF(J45&lt;=0,"Cycle must be above zero",IF(AND(J42&lt;&gt;"",J16&lt;&gt;0,J42&gt;J41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(J42&lt;&gt;"",J15&gt;0,J42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(J42="",J16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(J28=0,OR(J12&lt;&gt;0,_xlfn.ISFORMULA(J12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="K76" s="63">
+        <f>IF(K47&gt;1,"Close rate above 100%: not possible",IF(K45&lt;=0,"Cycle must be above zero",IF(AND(K42&lt;&gt;"",K16&lt;&gt;0,K42&gt;K41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(K42&lt;&gt;"",K15&gt;0,K42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(K42="",K16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(K28=0,OR(K12&lt;&gt;0,_xlfn.ISFORMULA(K12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="L76" s="63">
+        <f>IF(L47&gt;1,"Close rate above 100%: not possible",IF(L45&lt;=0,"Cycle must be above zero",IF(AND(L42&lt;&gt;"",L16&lt;&gt;0,L42&gt;L41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(L42&lt;&gt;"",L15&gt;0,L42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(L42="",L16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(L28=0,OR(L12&lt;&gt;0,_xlfn.ISFORMULA(L12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+      <c r="M76" s="63">
+        <f>IF(M47&gt;1,"Close rate above 100%: not possible",IF(M45&lt;=0,"Cycle must be above zero",IF(AND(M42&lt;&gt;"",M16&lt;&gt;0,M42&gt;M41),"Salespeople would hold more than they can manage: the extra opportunities are not worked",IF(AND(M42&lt;&gt;"",M15&gt;0,M42&lt;=v_opportunities_capacity),"Capacity increase has no effect: salespeople already hold fewer opportunities than they can manage",IF(AND(M42="",M16&lt;&gt;0),"No pipeline data on tab 1: this change has no effect until opportunities held is entered",IF(AND(M28=0,OR(M12&lt;&gt;0,_xlfn.ISFORMULA(M12))),"No open territories entered on tab 1 yet: this change has no effect","OK"))))))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:M2"/>
+  </mergeCells>
+  <conditionalFormatting sqref="D71:M71">
+    <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
+      <formula>"Balanced"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="2" operator="equal" dxfId="1">
+      <formula>"Check"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D76:M76">
+    <cfRule type="expression" priority="3" dxfId="1">
+      <formula>D76&lt;&gt;"OK"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="2">
+    <dataValidation sqref="B4" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Year one,Steady state"</formula1>
+    </dataValidation>
+    <dataValidation sqref="B5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>$E$7:$M$7</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
 </file>
</xml_diff>